<commit_message>
Incrementation add, readme, technical note.
</commit_message>
<xml_diff>
--- a/OTNOC_config.xlsx
+++ b/OTNOC_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Otnoc_Grafana_Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F189C64D-71CE-4A3E-B28F-95357FF953AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73403E96-5854-453F-BAFE-3D22448D7BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="9892" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51720" yWindow="-1695" windowWidth="51840" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
   <si>
     <t>Paramètre</t>
   </si>
@@ -319,118 +319,121 @@
     <t>Compteur OTNOC général ligne 3</t>
   </si>
   <si>
-    <t>OTNOC 2</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU1.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU2.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU3.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU4.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU5.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU6.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU7.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU8.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU9.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU10.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU11.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F3.AU12.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC1_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC2_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC3_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC4_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC5_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC6_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC7_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC8_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC9_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC10_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC11_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC12_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC13_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC14_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC15_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC16_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC17_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC18_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC19_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC20_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC21_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC22_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC23_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC24_F3.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC25_F3.DEF.PVFL</t>
+    <t>OTNOC</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU1.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU2.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU3.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU4.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU5.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU6.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU7.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU8.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU9.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU10.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU11.PVFL</t>
+  </si>
+  <si>
+    <t>AU_MEM_F1.AU12.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC1_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC2_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC3_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC4_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC5_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC6_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC7_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC8_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC9_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC10_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC11_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC12_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC13_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC14_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC15_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC16_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC17_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC18_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC19_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC20_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC21_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC22_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC23_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC24_F1.DEF.PVFL</t>
+  </si>
+  <si>
+    <t>OTNOC25_F1.DEF.PVFL</t>
   </si>
 </sst>
 </file>
@@ -848,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -903,6 +906,11 @@
       <c r="A6" s="2"/>
       <c r="B6" s="3"/>
       <c r="C6" s="4"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.4">
+      <c r="C33" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -933,7 +941,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
@@ -944,7 +952,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="9">
         <v>2</v>
@@ -955,7 +963,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" s="9">
         <v>3</v>
@@ -966,7 +974,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B5" s="9">
         <v>4</v>
@@ -977,7 +985,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6" s="9">
         <v>5</v>
@@ -988,7 +996,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B7" s="9">
         <v>6</v>
@@ -999,7 +1007,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B8" s="9">
         <v>7</v>
@@ -1010,7 +1018,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B9" s="9">
         <v>8</v>
@@ -1021,7 +1029,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B10" s="9">
         <v>9</v>
@@ -1032,7 +1040,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B11" s="9">
         <v>10</v>
@@ -1043,7 +1051,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" s="9">
         <v>11</v>
@@ -1054,7 +1062,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B13" s="9">
         <v>12</v>
@@ -1065,7 +1073,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B14" s="9">
         <v>1</v>
@@ -1076,7 +1084,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B15" s="9">
         <v>2</v>
@@ -1087,7 +1095,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B16" s="9">
         <v>3</v>
@@ -1098,7 +1106,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B17" s="9">
         <v>4</v>
@@ -1109,7 +1117,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B18" s="9">
         <v>5</v>
@@ -1120,7 +1128,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B19" s="9">
         <v>6</v>
@@ -1131,7 +1139,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B20" s="9">
         <v>7</v>
@@ -1142,7 +1150,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B21" s="9">
         <v>8</v>
@@ -1153,7 +1161,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B22" s="9">
         <v>9</v>
@@ -1164,7 +1172,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B23" s="9">
         <v>10</v>
@@ -1175,7 +1183,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B24" s="9">
         <v>11</v>
@@ -1186,7 +1194,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B25" s="9">
         <v>12</v>
@@ -1197,7 +1205,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B26" s="9">
         <v>13</v>
@@ -1208,7 +1216,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B27" s="9">
         <v>14</v>
@@ -1219,7 +1227,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B28" s="9">
         <v>15</v>
@@ -1230,7 +1238,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B29" s="9">
         <v>16</v>
@@ -1241,7 +1249,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B30" s="9">
         <v>17</v>
@@ -1252,7 +1260,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B31" s="9">
         <v>18</v>
@@ -1263,7 +1271,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B32" s="9">
         <v>19</v>
@@ -1274,7 +1282,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B33" s="9">
         <v>20</v>
@@ -1285,7 +1293,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B34" s="9">
         <v>21</v>
@@ -1296,7 +1304,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B35" s="9">
         <v>22</v>
@@ -1307,7 +1315,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B36" s="9">
         <v>23</v>
@@ -1318,7 +1326,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B37" s="9">
         <v>24</v>
@@ -1329,7 +1337,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B38" s="9">
         <v>25</v>

</xml_diff>

<commit_message>
Bool error fix, desc add
</commit_message>
<xml_diff>
--- a/OTNOC_config.xlsx
+++ b/OTNOC_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Otnoc_Grafana_Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73403E96-5854-453F-BAFE-3D22448D7BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD7F480-1675-41B2-B720-F1ED54461168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51720" yWindow="-1695" windowWidth="51840" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="44880" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
   <si>
     <t>Paramètre</t>
   </si>
@@ -130,24 +130,6 @@
     <t>text</t>
   </si>
   <si>
-    <t>Arrêt séquence ou défaut alimenteur</t>
-  </si>
-  <si>
-    <t>Arrêt séquence ou défaut grille</t>
-  </si>
-  <si>
-    <t>Arrêt ventilateur air primaire</t>
-  </si>
-  <si>
-    <t>Arrêt séquence ou défaut extracteur machefers</t>
-  </si>
-  <si>
-    <t>Défaut mesures O2 sortie chaudière et cheminée</t>
-  </si>
-  <si>
-    <t>Défaut OTNOC non automatisé</t>
-  </si>
-  <si>
     <t>MODE D'EMPLOI</t>
   </si>
   <si>
@@ -223,217 +205,19 @@
     <t xml:space="preserve">   - Renseigner le nom du site, le titre du panel.</t>
   </si>
   <si>
-    <t>UVE_ST_SAULVE</t>
-  </si>
-  <si>
     <t>AU 1</t>
   </si>
   <si>
-    <t>AU 2</t>
-  </si>
-  <si>
-    <t>AU 3</t>
-  </si>
-  <si>
-    <t>AU 4</t>
-  </si>
-  <si>
-    <t>AU 5</t>
-  </si>
-  <si>
-    <t>AU 6</t>
-  </si>
-  <si>
-    <t>AU 7</t>
-  </si>
-  <si>
-    <t>AU 8</t>
-  </si>
-  <si>
-    <t>AU 9</t>
-  </si>
-  <si>
-    <t>AU 10</t>
-  </si>
-  <si>
-    <t>AU 11</t>
-  </si>
-  <si>
-    <t>AU 12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surpression four </t>
-  </si>
-  <si>
-    <t>Arret ventilateur air secondaire</t>
-  </si>
-  <si>
-    <t>Défaut Brûleur et T2S seuil bas</t>
-  </si>
-  <si>
-    <t>O2 chaudière &gt; 10%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Température SCR infrieure au seuil limite </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Défaut des deux pompes injection urée </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Température entré FAM haute </t>
-  </si>
-  <si>
-    <t>Défaut champs électrofiltre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta P FAM très haute et niveau très haut sur 1 caisson </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pas d'injection bicar </t>
-  </si>
-  <si>
-    <t>Pas de soufflante injection réactifs</t>
-  </si>
-  <si>
-    <t>Défaut ou arret ventilateur de tirage</t>
-  </si>
-  <si>
-    <t>Pression air comprimé très basse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Défaut des deux vis d'injection de coke de lignite </t>
-  </si>
-  <si>
-    <t>Défaut dévouteur coke de lignite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase transitoire sans déchets si arret fortuit </t>
-  </si>
-  <si>
-    <t>Démarrage phase 2</t>
-  </si>
-  <si>
-    <t>Arret phase 1</t>
-  </si>
-  <si>
-    <t>Compteur OTNOC général ligne 3</t>
-  </si>
-  <si>
     <t>OTNOC</t>
   </si>
   <si>
     <t>x</t>
   </si>
   <si>
-    <t>AU_MEM_F1.AU1.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU2.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU3.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU4.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU5.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU6.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU7.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU8.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU9.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU10.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU11.PVFL</t>
-  </si>
-  <si>
-    <t>AU_MEM_F1.AU12.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC1_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC2_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC3_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC4_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC5_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC6_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC7_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC8_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC9_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC10_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC11_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC12_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC13_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC14_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC15_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC16_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC17_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC18_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC19_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC20_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC21_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC22_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC23_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC24_F1.DEF.PVFL</t>
-  </si>
-  <si>
-    <t>OTNOC25_F1.DEF.PVFL</t>
+    <t>AU_MEM_F2.AU1.PVFL</t>
+  </si>
+  <si>
+    <t>UVE_</t>
   </si>
 </sst>
 </file>
@@ -875,7 +659,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>4</v>
@@ -886,7 +670,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>6</v>
@@ -909,7 +693,7 @@
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.4">
       <c r="C33" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -941,410 +725,194 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="9">
-        <v>2</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>43</v>
-      </c>
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="8"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="9">
-        <v>3</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>44</v>
-      </c>
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="8"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="9">
-        <v>4</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>45</v>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="8"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="9">
-        <v>5</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>46</v>
-      </c>
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="8"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="9">
-        <v>6</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>47</v>
-      </c>
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="8"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B8" s="9">
-        <v>7</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>48</v>
-      </c>
+      <c r="A8" s="8"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="8"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="9">
-        <v>8</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>49</v>
-      </c>
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="8"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B10" s="9">
-        <v>9</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="A10" s="8"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="8"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="9">
-        <v>10</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>51</v>
-      </c>
+      <c r="A11" s="8"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="8"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="9">
-        <v>11</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>52</v>
-      </c>
+      <c r="A12" s="8"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="8"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="9">
-        <v>12</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>53</v>
-      </c>
+      <c r="A13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="8"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="9">
-        <v>1</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>10</v>
-      </c>
+      <c r="A14" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="8"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A15" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B15" s="9">
-        <v>2</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>54</v>
-      </c>
+      <c r="A15" s="8"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="8"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A16" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="9">
-        <v>3</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>11</v>
-      </c>
+      <c r="A16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A17" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="9">
-        <v>4</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="A17" s="8"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="8"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A18" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="9">
-        <v>5</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>55</v>
-      </c>
+      <c r="A18" s="8"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="8"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="9">
-        <v>6</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>56</v>
-      </c>
+      <c r="A19" s="8"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="8"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A20" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B20" s="9">
-        <v>7</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>13</v>
-      </c>
+      <c r="A20" s="8"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="8"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A21" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B21" s="9">
-        <v>8</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>14</v>
-      </c>
+      <c r="A21" s="8"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="8"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A22" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="9">
-        <v>9</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>57</v>
-      </c>
+      <c r="A22" s="8"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="8"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A23" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B23" s="9">
-        <v>10</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>58</v>
-      </c>
+      <c r="A23" s="8"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="8"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A24" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="9">
-        <v>11</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>59</v>
-      </c>
+      <c r="A24" s="8"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="8"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A25" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="9">
-        <v>12</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>60</v>
-      </c>
+      <c r="A25" s="8"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="8"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A26" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B26" s="9">
-        <v>13</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>61</v>
-      </c>
+      <c r="A26" s="8"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="8"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A27" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B27" s="9">
-        <v>14</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="A27" s="8"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="8"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A28" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B28" s="9">
-        <v>15</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>63</v>
-      </c>
+      <c r="A28" s="8"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="8"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A29" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B29" s="9">
-        <v>16</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>64</v>
-      </c>
+      <c r="A29" s="8"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="8"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A30" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B30" s="9">
-        <v>17</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>65</v>
-      </c>
+      <c r="A30" s="8"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="8"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A31" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="B31" s="9">
-        <v>18</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="A31" s="8"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="8"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A32" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B32" s="9">
-        <v>19</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>67</v>
-      </c>
+      <c r="A32" s="8"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="8"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A33" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B33" s="9">
-        <v>20</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>68</v>
-      </c>
+      <c r="A33" s="8"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="8"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A34" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B34" s="9">
-        <v>21</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>69</v>
-      </c>
+      <c r="A34" s="8"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="8"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A35" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B35" s="9">
-        <v>22</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>70</v>
-      </c>
+      <c r="A35" s="8"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="8"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A36" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B36" s="9">
-        <v>23</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>71</v>
-      </c>
+      <c r="A36" s="8"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="8"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A37" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B37" s="9">
-        <v>24</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>15</v>
-      </c>
+      <c r="A37" s="8"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="8"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A38" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B38" s="9">
-        <v>25</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>72</v>
-      </c>
+      <c r="A38" s="8"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1362,7 +930,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.4">
@@ -1370,17 +938,17 @@
     </row>
     <row r="3" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.4">
@@ -1388,37 +956,37 @@
     </row>
     <row r="7" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A7" s="5" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.4">
@@ -1426,42 +994,42 @@
     </row>
     <row r="15" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A15" s="5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" s="6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.4">
@@ -1469,37 +1037,37 @@
     </row>
     <row r="24" spans="1:1" ht="15.45" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A29" s="7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A30" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>